<commit_message>
3 scenarios working parallel with excel
</commit_message>
<xml_diff>
--- a/test-data/QA/TestData.xlsx
+++ b/test-data/QA/TestData.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\PLDemo\test-data\QA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8716F9AC-7AD0-4300-901C-58C296F3B1E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{55B4C4EE-E40D-43EA-97BB-2C4D9A7C53A6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{E9EE1CF9-2DBE-4411-BB3C-108DF62B0878}"/>
   </bookViews>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="31">
   <si>
     <t>TestCase</t>
   </si>
@@ -78,12 +78,6 @@
     <t>Create New Contact</t>
   </si>
   <si>
-    <t>Nikhil</t>
-  </si>
-  <si>
-    <t>Patil</t>
-  </si>
-  <si>
     <t>Birth_Day</t>
   </si>
   <si>
@@ -109,6 +103,24 @@
   </si>
   <si>
     <t>Is_Do_not_Text</t>
+  </si>
+  <si>
+    <t>Vinit</t>
+  </si>
+  <si>
+    <t>Pathak</t>
+  </si>
+  <si>
+    <t>Delete Created New Contact</t>
+  </si>
+  <si>
+    <t>Sameer</t>
+  </si>
+  <si>
+    <t>TC0002</t>
+  </si>
+  <si>
+    <t>TC0011</t>
   </si>
 </sst>
 </file>
@@ -490,7 +502,7 @@
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="15" customWidth="1"/>
-    <col min="2" max="2" width="17.6640625" customWidth="1"/>
+    <col min="2" max="2" width="30.21875" customWidth="1"/>
     <col min="3" max="4" width="13.44140625" customWidth="1"/>
     <col min="5" max="5" width="10.88671875" customWidth="1"/>
     <col min="7" max="7" width="13.44140625" customWidth="1"/>
@@ -503,7 +515,7 @@
   <sheetData>
     <row r="1" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>1</v>
@@ -524,25 +536,25 @@
         <v>13</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="I1" s="1" t="s">
         <v>14</v>
       </c>
       <c r="J1" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="L1" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="M1" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="N1" s="1" t="s">
         <v>19</v>
-      </c>
-      <c r="L1" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="M1" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="N1" s="1" t="s">
-        <v>21</v>
       </c>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.3">
@@ -553,10 +565,10 @@
         <v>15</v>
       </c>
       <c r="C2" t="s">
-        <v>16</v>
+        <v>25</v>
       </c>
       <c r="D2" t="s">
-        <v>17</v>
+        <v>26</v>
       </c>
       <c r="E2" t="s">
         <v>10</v>
@@ -565,13 +577,13 @@
         <v>12</v>
       </c>
       <c r="G2" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="H2" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="I2" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="J2">
         <v>1</v>
@@ -583,14 +595,55 @@
         <v>1995</v>
       </c>
       <c r="M2" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="N2">
         <v>2</v>
       </c>
     </row>
     <row r="3" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="N3" s="1"/>
+      <c r="A3" t="s">
+        <v>29</v>
+      </c>
+      <c r="B3" t="s">
+        <v>27</v>
+      </c>
+      <c r="C3" t="s">
+        <v>28</v>
+      </c>
+      <c r="D3" t="s">
+        <v>26</v>
+      </c>
+      <c r="E3" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G3" t="s">
+        <v>22</v>
+      </c>
+      <c r="H3" t="s">
+        <v>22</v>
+      </c>
+      <c r="I3" t="s">
+        <v>22</v>
+      </c>
+      <c r="J3">
+        <v>1</v>
+      </c>
+      <c r="K3">
+        <v>5</v>
+      </c>
+      <c r="L3">
+        <v>1995</v>
+      </c>
+      <c r="M3" t="s">
+        <v>20</v>
+      </c>
+      <c r="N3">
+        <v>2</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -600,7 +653,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DB71EF1D-3515-439D-8923-EFE06D1ABB9D}">
-  <dimension ref="A1:H1"/>
+  <dimension ref="A1:H2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="3" max="3" width="12.109375" customWidth="1"/>
@@ -608,7 +661,7 @@
     <col min="5" max="5" width="10.21875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -632,6 +685,11 @@
       </c>
       <c r="H1" s="1" t="s">
         <v>7</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>30</v>
       </c>
     </row>
   </sheetData>

</xml_diff>